<commit_message>
Fig.7: compare v4 with CAT-37 (default) and CAT-50 (robust); CAT-47 kept as dashed reference (PNG/SVG + xlsx)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7.xlsx
+++ b/figs/data/fig7.xlsx
@@ -162,11 +162,83 @@
           <order val="0"/>
           <tx>
             <strRef>
+              <f>'OLTP→Varmail'!Q1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="E3A33B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$P$2:$P$60</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$Q$2:$Q$60</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'OLTP→Varmail'!S1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="8E8E93"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$R$2:$R$61</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$S$2:$S$61</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
               <f>'OLTP→Varmail'!D1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
               <a:solidFill>
                 <a:srgbClr val="1D1D1F"/>
               </a:solidFill>
@@ -194,15 +266,15 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="1"/>
-          <order val="1"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'OLTP→Varmail'!B1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="15875">
               <a:solidFill>
                 <a:srgbClr val="2A78D6"/>
               </a:solidFill>
@@ -230,11 +302,11 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
-              <f>'OLTP→Varmail'!T1</f>
+              <f>'OLTP→Varmail'!X1</f>
             </strRef>
           </tx>
           <spPr>
@@ -255,12 +327,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$S$2:$S$3</f>
+              <f>'OLTP→Varmail'!$W$2:$W$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$T$2:$T$3</f>
+              <f>'OLTP→Varmail'!$X$2:$X$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -302,8 +374,8 @@
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="2.1"/>
-          <min val="1.2"/>
+          <max val="30.1"/>
+          <min val="0.5"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -400,7 +472,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'OLTP→Varmail'!V1</f>
+              <f>'OLTP→Varmail'!Z1</f>
             </strRef>
           </tx>
           <spPr>
@@ -421,12 +493,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$U$2:$U$3</f>
+              <f>'OLTP→Varmail'!$Y$2:$Y$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$V$2:$V$3</f>
+              <f>'OLTP→Varmail'!$Z$2:$Z$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -566,7 +638,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'OLTP→Varmail'!X1</f>
+              <f>'OLTP→Varmail'!AB1</f>
             </strRef>
           </tx>
           <spPr>
@@ -587,12 +659,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$W$2:$W$3</f>
+              <f>'OLTP→Varmail'!$AA$2:$AA$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$X$2:$X$3</f>
+              <f>'OLTP→Varmail'!$AB$2:$AB$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -696,11 +768,83 @@
           <order val="0"/>
           <tx>
             <strRef>
+              <f>'FIO-Fast→Varmail'!Q1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="E3A33B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$P$2:$P$90</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$Q$2:$Q$90</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'FIO-Fast→Varmail'!S1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22225">
+              <a:solidFill>
+                <a:srgbClr val="8E8E93"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$R$2:$R$90</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$S$2:$S$90</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
               <f>'FIO-Fast→Varmail'!D1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
               <a:solidFill>
                 <a:srgbClr val="1D1D1F"/>
               </a:solidFill>
@@ -728,15 +872,15 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="1"/>
-          <order val="1"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'FIO-Fast→Varmail'!B1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="15875">
               <a:solidFill>
                 <a:srgbClr val="2A78D6"/>
               </a:solidFill>
@@ -764,11 +908,11 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
-              <f>'FIO-Fast→Varmail'!T1</f>
+              <f>'FIO-Fast→Varmail'!X1</f>
             </strRef>
           </tx>
           <spPr>
@@ -789,12 +933,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$S$2:$S$3</f>
+              <f>'FIO-Fast→Varmail'!$W$2:$W$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$T$2:$T$3</f>
+              <f>'FIO-Fast→Varmail'!$X$2:$X$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -836,8 +980,8 @@
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="3.8"/>
-          <min val="1.6"/>
+          <max val="44.6"/>
+          <min val="0.5"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -934,7 +1078,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'FIO-Fast→Varmail'!V1</f>
+              <f>'FIO-Fast→Varmail'!Z1</f>
             </strRef>
           </tx>
           <spPr>
@@ -955,12 +1099,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$U$2:$U$3</f>
+              <f>'FIO-Fast→Varmail'!$Y$2:$Y$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$V$2:$V$3</f>
+              <f>'FIO-Fast→Varmail'!$Z$2:$Z$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -1100,7 +1244,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'FIO-Fast→Varmail'!X1</f>
+              <f>'FIO-Fast→Varmail'!AB1</f>
             </strRef>
           </tx>
           <spPr>
@@ -1121,12 +1265,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$W$2:$W$3</f>
+              <f>'FIO-Fast→Varmail'!$AA$2:$AA$3</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'FIO-Fast→Varmail'!$X$2:$X$3</f>
+              <f>'FIO-Fast→Varmail'!$AB$2:$AB$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -1207,7 +1351,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1229,7 +1373,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -1251,7 +1395,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>39</row>
       <rowOff>0</rowOff>
@@ -1278,7 +1422,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1300,7 +1444,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>20</row>
       <rowOff>0</rowOff>
@@ -1322,7 +1466,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>25</col>
+      <col>29</col>
       <colOff>0</colOff>
       <row>39</row>
       <rowOff>0</rowOff>
@@ -1634,7 +1778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X676"/>
+  <dimension ref="A1:AB676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1652,6 +1796,10 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1730,37 +1878,57 @@
           <t>학습 상태 (0=전수 순회, 1=탐색, 2=정착)</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-37 시간(분)</t>
+        </is>
+      </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>CAT-37 (기본) 30초 WAF</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-50 시간(분)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-50 (견고) 30초 WAF</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>전환 시점(분)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>워크로드 전환 (16.0분)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>워크로드 전환 (16.0분)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>워크로드 전환 (16.0분)</t>
         </is>
@@ -1812,25 +1980,37 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
+      <c r="P2" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Q2" t="n">
-        <v>16.02</v>
+        <v>1.5039</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.5</v>
       </c>
       <c r="S2" t="n">
-        <v>16.02</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1.2</v>
+        <v>1.4228</v>
       </c>
       <c r="U2" t="n">
         <v>16.02</v>
       </c>
-      <c r="V2" t="n">
-        <v>-0.2</v>
-      </c>
       <c r="W2" t="n">
         <v>16.02</v>
       </c>
       <c r="X2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="AB2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1880,27 +2060,39 @@
       <c r="O3" t="n">
         <v>0</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.3942</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1.252</v>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>※ 각 열 쌍(시간, 값)이 그래프의 선 하나. 색·굵기·제목은 차트를 클릭해서 수정.</t>
         </is>
-      </c>
-      <c r="S3" t="n">
-        <v>16.02</v>
-      </c>
-      <c r="T3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>16.02</v>
-      </c>
-      <c r="V3" t="n">
-        <v>2.2</v>
       </c>
       <c r="W3" t="n">
         <v>16.02</v>
       </c>
       <c r="X3" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="AB3" t="n">
         <v>48</v>
       </c>
     </row>
@@ -1950,6 +2142,18 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
+      <c r="P4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1.3698</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1.2599</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1997,6 +2201,18 @@
       <c r="O5" t="n">
         <v>0</v>
       </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1.3353</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1.2642</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2044,6 +2260,18 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
+      <c r="P6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.342</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1.2519</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2091,6 +2319,18 @@
       <c r="O7" t="n">
         <v>0</v>
       </c>
+      <c r="P7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1.3496</v>
+      </c>
+      <c r="R7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1.2544</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2138,6 +2378,18 @@
       <c r="O8" t="n">
         <v>0</v>
       </c>
+      <c r="P8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1.3366</v>
+      </c>
+      <c r="R8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1.2446</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2185,6 +2437,18 @@
       <c r="O9" t="n">
         <v>0</v>
       </c>
+      <c r="P9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1.337</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.2382</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2232,6 +2496,18 @@
       <c r="O10" t="n">
         <v>0</v>
       </c>
+      <c r="P10" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1.3359</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1.2398</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2279,6 +2555,18 @@
       <c r="O11" t="n">
         <v>0</v>
       </c>
+      <c r="P11" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1.3295</v>
+      </c>
+      <c r="R11" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1.2383</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2326,6 +2614,18 @@
       <c r="O12" t="n">
         <v>0</v>
       </c>
+      <c r="P12" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1.3298</v>
+      </c>
+      <c r="R12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1.2447</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2373,6 +2673,18 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
+      <c r="P13" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1.3327</v>
+      </c>
+      <c r="R13" t="n">
+        <v>6</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1.2351</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2420,6 +2732,18 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
+      <c r="P14" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1.3259</v>
+      </c>
+      <c r="R14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="S14" t="n">
+        <v>1.2379</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2467,6 +2791,18 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
+      <c r="P15" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.3205</v>
+      </c>
+      <c r="R15" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1.2358</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2514,6 +2850,18 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
+      <c r="P16" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1.3235</v>
+      </c>
+      <c r="R16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1.2344</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2561,6 +2909,18 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
+      <c r="P17" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1.321</v>
+      </c>
+      <c r="R17" t="n">
+        <v>8</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1.2365</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2608,6 +2968,18 @@
       <c r="O18" t="n">
         <v>0</v>
       </c>
+      <c r="P18" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1.3205</v>
+      </c>
+      <c r="R18" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1.2387</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2655,6 +3027,18 @@
       <c r="O19" t="n">
         <v>0</v>
       </c>
+      <c r="P19" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1.3189</v>
+      </c>
+      <c r="R19" t="n">
+        <v>9</v>
+      </c>
+      <c r="S19" t="n">
+        <v>1.2386</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2702,6 +3086,18 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
+      <c r="P20" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1.3187</v>
+      </c>
+      <c r="R20" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="S20" t="n">
+        <v>1.2353</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2749,6 +3145,18 @@
       <c r="O21" t="n">
         <v>0</v>
       </c>
+      <c r="P21" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1.3128</v>
+      </c>
+      <c r="R21" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="S21" t="n">
+        <v>1.2363</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2796,6 +3204,18 @@
       <c r="O22" t="n">
         <v>0</v>
       </c>
+      <c r="P22" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1.3155</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="S22" t="n">
+        <v>1.2377</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2843,6 +3263,18 @@
       <c r="O23" t="n">
         <v>0</v>
       </c>
+      <c r="P23" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="R23" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="S23" t="n">
+        <v>1.2403</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2890,6 +3322,18 @@
       <c r="O24" t="n">
         <v>0</v>
       </c>
+      <c r="P24" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1.3137</v>
+      </c>
+      <c r="R24" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="S24" t="n">
+        <v>1.2405</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2937,6 +3381,18 @@
       <c r="O25" t="n">
         <v>0</v>
       </c>
+      <c r="P25" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1.3136</v>
+      </c>
+      <c r="R25" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1.2409</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2984,6 +3440,18 @@
       <c r="O26" t="n">
         <v>0</v>
       </c>
+      <c r="P26" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1.3123</v>
+      </c>
+      <c r="R26" t="n">
+        <v>12.52</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.2405</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3031,6 +3499,18 @@
       <c r="O27" t="n">
         <v>0</v>
       </c>
+      <c r="P27" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="R27" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="S27" t="n">
+        <v>1.2425</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3078,6 +3558,18 @@
       <c r="O28" t="n">
         <v>0</v>
       </c>
+      <c r="P28" t="n">
+        <v>13.55</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1.3113</v>
+      </c>
+      <c r="R28" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="S28" t="n">
+        <v>1.242</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3125,6 +3617,18 @@
       <c r="O29" t="n">
         <v>0</v>
       </c>
+      <c r="P29" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>1.3101</v>
+      </c>
+      <c r="R29" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="S29" t="n">
+        <v>1.2423</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3172,6 +3676,18 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
+      <c r="P30" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>1.3111</v>
+      </c>
+      <c r="R30" t="n">
+        <v>14.52</v>
+      </c>
+      <c r="S30" t="n">
+        <v>1.244</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3219,6 +3735,18 @@
       <c r="O31" t="n">
         <v>0</v>
       </c>
+      <c r="P31" t="n">
+        <v>15.05</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>1.3606</v>
+      </c>
+      <c r="R31" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="S31" t="n">
+        <v>1.2454</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3266,6 +3794,18 @@
       <c r="O32" t="n">
         <v>0</v>
       </c>
+      <c r="P32" t="n">
+        <v>15.55</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>2.1374</v>
+      </c>
+      <c r="R32" t="n">
+        <v>15.52</v>
+      </c>
+      <c r="S32" t="n">
+        <v>1.5873</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3313,6 +3853,18 @@
       <c r="O33" t="n">
         <v>0</v>
       </c>
+      <c r="P33" t="n">
+        <v>16.05</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>2.3831</v>
+      </c>
+      <c r="R33" t="n">
+        <v>16.02</v>
+      </c>
+      <c r="S33" t="n">
+        <v>2.0166</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3360,6 +3912,18 @@
       <c r="O34" t="n">
         <v>0</v>
       </c>
+      <c r="P34" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>2.3912</v>
+      </c>
+      <c r="R34" t="n">
+        <v>16.52</v>
+      </c>
+      <c r="S34" t="n">
+        <v>2.064</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3407,6 +3971,18 @@
       <c r="O35" t="n">
         <v>0</v>
       </c>
+      <c r="P35" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>2.3943</v>
+      </c>
+      <c r="R35" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="S35" t="n">
+        <v>2.0791</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3454,6 +4030,18 @@
       <c r="O36" t="n">
         <v>0</v>
       </c>
+      <c r="P36" t="n">
+        <v>17.55</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>2.4031</v>
+      </c>
+      <c r="R36" t="n">
+        <v>17.52</v>
+      </c>
+      <c r="S36" t="n">
+        <v>2.0877</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3501,6 +4089,18 @@
       <c r="O37" t="n">
         <v>0</v>
       </c>
+      <c r="P37" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>2.4016</v>
+      </c>
+      <c r="R37" t="n">
+        <v>18.02</v>
+      </c>
+      <c r="S37" t="n">
+        <v>2.0921</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3548,6 +4148,18 @@
       <c r="O38" t="n">
         <v>0</v>
       </c>
+      <c r="P38" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>2.4026</v>
+      </c>
+      <c r="R38" t="n">
+        <v>18.52</v>
+      </c>
+      <c r="S38" t="n">
+        <v>2.0911</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3595,6 +4207,18 @@
       <c r="O39" t="n">
         <v>0</v>
       </c>
+      <c r="P39" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>2.4054</v>
+      </c>
+      <c r="R39" t="n">
+        <v>19.02</v>
+      </c>
+      <c r="S39" t="n">
+        <v>2.092</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3642,6 +4266,18 @@
       <c r="O40" t="n">
         <v>0</v>
       </c>
+      <c r="P40" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>2.405</v>
+      </c>
+      <c r="R40" t="n">
+        <v>19.52</v>
+      </c>
+      <c r="S40" t="n">
+        <v>2.0954</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3689,6 +4325,18 @@
       <c r="O41" t="n">
         <v>0</v>
       </c>
+      <c r="P41" t="n">
+        <v>20.05</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.4048</v>
+      </c>
+      <c r="R41" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.0912</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3736,6 +4384,18 @@
       <c r="O42" t="n">
         <v>0</v>
       </c>
+      <c r="P42" t="n">
+        <v>20.55</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>2.4002</v>
+      </c>
+      <c r="R42" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="S42" t="n">
+        <v>2.0949</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3783,6 +4443,18 @@
       <c r="O43" t="n">
         <v>0</v>
       </c>
+      <c r="P43" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>2.3995</v>
+      </c>
+      <c r="R43" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="S43" t="n">
+        <v>2.0925</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3830,6 +4502,18 @@
       <c r="O44" t="n">
         <v>0</v>
       </c>
+      <c r="P44" t="n">
+        <v>21.55</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.4031</v>
+      </c>
+      <c r="R44" t="n">
+        <v>21.52</v>
+      </c>
+      <c r="S44" t="n">
+        <v>2.0908</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3877,6 +4561,18 @@
       <c r="O45" t="n">
         <v>0</v>
       </c>
+      <c r="P45" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>2.4055</v>
+      </c>
+      <c r="R45" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="S45" t="n">
+        <v>2.0952</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3928,6 +4624,18 @@
       <c r="O46" t="n">
         <v>0</v>
       </c>
+      <c r="P46" t="n">
+        <v>22.55</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>2.4029</v>
+      </c>
+      <c r="R46" t="n">
+        <v>22.52</v>
+      </c>
+      <c r="S46" t="n">
+        <v>2.0957</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3979,6 +4687,18 @@
       <c r="O47" t="n">
         <v>0</v>
       </c>
+      <c r="P47" t="n">
+        <v>23.05</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.3994</v>
+      </c>
+      <c r="R47" t="n">
+        <v>23.02</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.0964</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4030,6 +4750,18 @@
       <c r="O48" t="n">
         <v>0</v>
       </c>
+      <c r="P48" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.4022</v>
+      </c>
+      <c r="R48" t="n">
+        <v>23.52</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.0967</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4081,6 +4813,18 @@
       <c r="O49" t="n">
         <v>0</v>
       </c>
+      <c r="P49" t="n">
+        <v>24.05</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.3991</v>
+      </c>
+      <c r="R49" t="n">
+        <v>24.02</v>
+      </c>
+      <c r="S49" t="n">
+        <v>2.0933</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4132,6 +4876,18 @@
       <c r="O50" t="n">
         <v>0</v>
       </c>
+      <c r="P50" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>2.4022</v>
+      </c>
+      <c r="R50" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="S50" t="n">
+        <v>2.0991</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4183,6 +4939,18 @@
       <c r="O51" t="n">
         <v>0</v>
       </c>
+      <c r="P51" t="n">
+        <v>25.05</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>2.3952</v>
+      </c>
+      <c r="R51" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="S51" t="n">
+        <v>2.0941</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4234,6 +5002,18 @@
       <c r="O52" t="n">
         <v>0</v>
       </c>
+      <c r="P52" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>2.3941</v>
+      </c>
+      <c r="R52" t="n">
+        <v>25.52</v>
+      </c>
+      <c r="S52" t="n">
+        <v>2.0977</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4285,6 +5065,18 @@
       <c r="O53" t="n">
         <v>0</v>
       </c>
+      <c r="P53" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>2.393</v>
+      </c>
+      <c r="R53" t="n">
+        <v>26.02</v>
+      </c>
+      <c r="S53" t="n">
+        <v>2.0948</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4336,6 +5128,18 @@
       <c r="O54" t="n">
         <v>0</v>
       </c>
+      <c r="P54" t="n">
+        <v>26.55</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>2.3941</v>
+      </c>
+      <c r="R54" t="n">
+        <v>26.52</v>
+      </c>
+      <c r="S54" t="n">
+        <v>2.0951</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4387,6 +5191,18 @@
       <c r="O55" t="n">
         <v>0</v>
       </c>
+      <c r="P55" t="n">
+        <v>27.05</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>2.3876</v>
+      </c>
+      <c r="R55" t="n">
+        <v>27.02</v>
+      </c>
+      <c r="S55" t="n">
+        <v>2.1033</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4438,6 +5254,18 @@
       <c r="O56" t="n">
         <v>0</v>
       </c>
+      <c r="P56" t="n">
+        <v>27.55</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>2.3897</v>
+      </c>
+      <c r="R56" t="n">
+        <v>27.52</v>
+      </c>
+      <c r="S56" t="n">
+        <v>2.1016</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4489,6 +5317,18 @@
       <c r="O57" t="n">
         <v>0</v>
       </c>
+      <c r="P57" t="n">
+        <v>28.05</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>2.3909</v>
+      </c>
+      <c r="R57" t="n">
+        <v>28.02</v>
+      </c>
+      <c r="S57" t="n">
+        <v>2.0993</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4540,6 +5380,18 @@
       <c r="O58" t="n">
         <v>0</v>
       </c>
+      <c r="P58" t="n">
+        <v>28.55</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>2.3889</v>
+      </c>
+      <c r="R58" t="n">
+        <v>28.52</v>
+      </c>
+      <c r="S58" t="n">
+        <v>2.0936</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4591,6 +5443,18 @@
       <c r="O59" t="n">
         <v>0</v>
       </c>
+      <c r="P59" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>2.3873</v>
+      </c>
+      <c r="R59" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="S59" t="n">
+        <v>2.0977</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4642,6 +5506,18 @@
       <c r="O60" t="n">
         <v>0</v>
       </c>
+      <c r="P60" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>2.3866</v>
+      </c>
+      <c r="R60" t="n">
+        <v>29.52</v>
+      </c>
+      <c r="S60" t="n">
+        <v>2.0965</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4686,6 +5562,12 @@
       </c>
       <c r="O61" t="n">
         <v>0</v>
+      </c>
+      <c r="R61" t="n">
+        <v>30.02</v>
+      </c>
+      <c r="S61" t="n">
+        <v>2.0966</v>
       </c>
     </row>
     <row r="62">
@@ -23066,7 +23948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X648"/>
+  <dimension ref="A1:AB648"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23084,6 +23966,10 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23162,37 +24048,57 @@
           <t>학습 상태 (0=전수 순회, 1=탐색, 2=정착)</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-37 시간(분)</t>
+        </is>
+      </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>CAT-37 (기본) 30초 WAF</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-50 시간(분)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-50 (견고) 30초 WAF</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>전환 시점(분)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>워크로드 전환 (30.1분)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>워크로드 전환 (30.1분)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>전환 시간</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>워크로드 전환 (30.1분)</t>
         </is>
@@ -23244,25 +24150,37 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
+      <c r="P2" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Q2" t="n">
-        <v>30.05</v>
+        <v>1.93</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.5</v>
       </c>
       <c r="S2" t="n">
-        <v>30.05</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1.6</v>
+        <v>1.8786</v>
       </c>
       <c r="U2" t="n">
         <v>30.05</v>
       </c>
-      <c r="V2" t="n">
-        <v>-0.2</v>
-      </c>
       <c r="W2" t="n">
         <v>30.05</v>
       </c>
       <c r="X2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="AB2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -23312,27 +24230,39 @@
       <c r="O3" t="n">
         <v>0</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1.9474</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1.7846</v>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>※ 각 열 쌍(시간, 값)이 그래프의 선 하나. 색·굵기·제목은 차트를 클릭해서 수정.</t>
         </is>
-      </c>
-      <c r="S3" t="n">
-        <v>30.05</v>
-      </c>
-      <c r="T3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="U3" t="n">
-        <v>30.05</v>
-      </c>
-      <c r="V3" t="n">
-        <v>2.2</v>
       </c>
       <c r="W3" t="n">
         <v>30.05</v>
       </c>
       <c r="X3" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>30.05</v>
+      </c>
+      <c r="AB3" t="n">
         <v>48</v>
       </c>
     </row>
@@ -23382,6 +24312,18 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
+      <c r="P4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1.9714</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1.8714</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -23429,6 +24371,18 @@
       <c r="O5" t="n">
         <v>0</v>
       </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2.0234</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1.8533</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -23476,6 +24430,18 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
+      <c r="P6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.9989</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1.837</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -23523,6 +24489,18 @@
       <c r="O7" t="n">
         <v>0</v>
       </c>
+      <c r="P7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1.9691</v>
+      </c>
+      <c r="R7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1.8062</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -23570,6 +24548,18 @@
       <c r="O8" t="n">
         <v>0</v>
       </c>
+      <c r="P8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1.961</v>
+      </c>
+      <c r="R8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1.7935</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -23617,6 +24607,18 @@
       <c r="O9" t="n">
         <v>0</v>
       </c>
+      <c r="P9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1.9097</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1.7624</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -23664,6 +24666,18 @@
       <c r="O10" t="n">
         <v>0</v>
       </c>
+      <c r="P10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1.8989</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1.7501</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -23711,6 +24725,18 @@
       <c r="O11" t="n">
         <v>0</v>
       </c>
+      <c r="P11" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1.902</v>
+      </c>
+      <c r="R11" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1.7748</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -23758,6 +24784,18 @@
       <c r="O12" t="n">
         <v>0</v>
       </c>
+      <c r="P12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>2.0439</v>
+      </c>
+      <c r="R12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1.8431</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -23805,6 +24843,18 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
+      <c r="P13" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>2.0325</v>
+      </c>
+      <c r="R13" t="n">
+        <v>6</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1.8658</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -23852,6 +24902,18 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
+      <c r="P14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>2.0317</v>
+      </c>
+      <c r="R14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="S14" t="n">
+        <v>1.8348</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -23899,6 +24961,18 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
+      <c r="P15" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.9836</v>
+      </c>
+      <c r="R15" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1.8316</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -23946,6 +25020,18 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
+      <c r="P16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1.9838</v>
+      </c>
+      <c r="R16" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1.8217</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -23993,6 +25079,18 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
+      <c r="P17" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1.9433</v>
+      </c>
+      <c r="R17" t="n">
+        <v>8</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1.8087</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -24040,6 +25138,18 @@
       <c r="O18" t="n">
         <v>0</v>
       </c>
+      <c r="P18" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1.9324</v>
+      </c>
+      <c r="R18" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1.7856</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -24087,6 +25197,18 @@
       <c r="O19" t="n">
         <v>0</v>
       </c>
+      <c r="P19" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1.9102</v>
+      </c>
+      <c r="R19" t="n">
+        <v>9</v>
+      </c>
+      <c r="S19" t="n">
+        <v>1.7559</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -24134,6 +25256,18 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
+      <c r="P20" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1.9607</v>
+      </c>
+      <c r="R20" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="S20" t="n">
+        <v>1.7962</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -24181,6 +25315,18 @@
       <c r="O21" t="n">
         <v>0</v>
       </c>
+      <c r="P21" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>2.0366</v>
+      </c>
+      <c r="R21" t="n">
+        <v>10</v>
+      </c>
+      <c r="S21" t="n">
+        <v>1.8252</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -24228,6 +25374,18 @@
       <c r="O22" t="n">
         <v>0</v>
       </c>
+      <c r="P22" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>2.0543</v>
+      </c>
+      <c r="R22" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="S22" t="n">
+        <v>1.8471</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -24275,6 +25433,18 @@
       <c r="O23" t="n">
         <v>0</v>
       </c>
+      <c r="P23" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1.9925</v>
+      </c>
+      <c r="R23" t="n">
+        <v>11</v>
+      </c>
+      <c r="S23" t="n">
+        <v>1.819</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -24322,6 +25492,18 @@
       <c r="O24" t="n">
         <v>0</v>
       </c>
+      <c r="P24" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1.988</v>
+      </c>
+      <c r="R24" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="S24" t="n">
+        <v>1.8235</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -24369,6 +25551,18 @@
       <c r="O25" t="n">
         <v>0</v>
       </c>
+      <c r="P25" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1.9428</v>
+      </c>
+      <c r="R25" t="n">
+        <v>12</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1.8178</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -24416,6 +25610,18 @@
       <c r="O26" t="n">
         <v>0</v>
       </c>
+      <c r="P26" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1.9507</v>
+      </c>
+      <c r="R26" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S26" t="n">
+        <v>1.7997</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -24463,6 +25669,18 @@
       <c r="O27" t="n">
         <v>0</v>
       </c>
+      <c r="P27" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1.9171</v>
+      </c>
+      <c r="R27" t="n">
+        <v>13</v>
+      </c>
+      <c r="S27" t="n">
+        <v>1.7858</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -24510,6 +25728,18 @@
       <c r="O28" t="n">
         <v>0</v>
       </c>
+      <c r="P28" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1.9148</v>
+      </c>
+      <c r="R28" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="S28" t="n">
+        <v>1.768</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -24557,6 +25787,18 @@
       <c r="O29" t="n">
         <v>0</v>
       </c>
+      <c r="P29" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>1.9916</v>
+      </c>
+      <c r="R29" t="n">
+        <v>14</v>
+      </c>
+      <c r="S29" t="n">
+        <v>1.8375</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -24604,6 +25846,18 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
+      <c r="P30" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>2.0625</v>
+      </c>
+      <c r="R30" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="S30" t="n">
+        <v>1.8569</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -24651,6 +25905,18 @@
       <c r="O31" t="n">
         <v>0</v>
       </c>
+      <c r="P31" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>2.0414</v>
+      </c>
+      <c r="R31" t="n">
+        <v>15</v>
+      </c>
+      <c r="S31" t="n">
+        <v>1.8333</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -24698,6 +25964,18 @@
       <c r="O32" t="n">
         <v>0</v>
       </c>
+      <c r="P32" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>2.0082</v>
+      </c>
+      <c r="R32" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="S32" t="n">
+        <v>1.8256</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -24745,6 +26023,18 @@
       <c r="O33" t="n">
         <v>0</v>
       </c>
+      <c r="P33" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>1.9734</v>
+      </c>
+      <c r="R33" t="n">
+        <v>16</v>
+      </c>
+      <c r="S33" t="n">
+        <v>1.7915</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -24792,6 +26082,18 @@
       <c r="O34" t="n">
         <v>0</v>
       </c>
+      <c r="P34" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1.9551</v>
+      </c>
+      <c r="R34" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="S34" t="n">
+        <v>1.8052</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -24839,6 +26141,18 @@
       <c r="O35" t="n">
         <v>0</v>
       </c>
+      <c r="P35" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1.9279</v>
+      </c>
+      <c r="R35" t="n">
+        <v>17</v>
+      </c>
+      <c r="S35" t="n">
+        <v>1.7748</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -24886,6 +26200,18 @@
       <c r="O36" t="n">
         <v>0</v>
       </c>
+      <c r="P36" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>1.8938</v>
+      </c>
+      <c r="R36" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="S36" t="n">
+        <v>1.7834</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -24933,6 +26259,18 @@
       <c r="O37" t="n">
         <v>0</v>
       </c>
+      <c r="P37" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>1.9203</v>
+      </c>
+      <c r="R37" t="n">
+        <v>18</v>
+      </c>
+      <c r="S37" t="n">
+        <v>1.7743</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -24980,6 +26318,18 @@
       <c r="O38" t="n">
         <v>0</v>
       </c>
+      <c r="P38" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>2.0321</v>
+      </c>
+      <c r="R38" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="S38" t="n">
+        <v>1.8407</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -25027,6 +26377,18 @@
       <c r="O39" t="n">
         <v>0</v>
       </c>
+      <c r="P39" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>2.064</v>
+      </c>
+      <c r="R39" t="n">
+        <v>19</v>
+      </c>
+      <c r="S39" t="n">
+        <v>1.8594</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -25074,6 +26436,18 @@
       <c r="O40" t="n">
         <v>0</v>
       </c>
+      <c r="P40" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>2.0293</v>
+      </c>
+      <c r="R40" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="S40" t="n">
+        <v>1.8536</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -25121,6 +26495,18 @@
       <c r="O41" t="n">
         <v>0</v>
       </c>
+      <c r="P41" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.0072</v>
+      </c>
+      <c r="R41" t="n">
+        <v>20</v>
+      </c>
+      <c r="S41" t="n">
+        <v>1.8426</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -25168,6 +26554,18 @@
       <c r="O42" t="n">
         <v>0</v>
       </c>
+      <c r="P42" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.9836</v>
+      </c>
+      <c r="R42" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.8162</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -25215,6 +26613,18 @@
       <c r="O43" t="n">
         <v>0</v>
       </c>
+      <c r="P43" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.9615</v>
+      </c>
+      <c r="R43" t="n">
+        <v>21</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.7893</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -25262,6 +26672,18 @@
       <c r="O44" t="n">
         <v>0</v>
       </c>
+      <c r="P44" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>1.921</v>
+      </c>
+      <c r="R44" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.7778</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -25309,6 +26731,18 @@
       <c r="O45" t="n">
         <v>0</v>
       </c>
+      <c r="P45" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.9038</v>
+      </c>
+      <c r="R45" t="n">
+        <v>22</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.737</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -25360,6 +26794,18 @@
       <c r="O46" t="n">
         <v>0</v>
       </c>
+      <c r="P46" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.929</v>
+      </c>
+      <c r="R46" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.7898</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -25411,6 +26857,18 @@
       <c r="O47" t="n">
         <v>0</v>
       </c>
+      <c r="P47" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.0382</v>
+      </c>
+      <c r="R47" t="n">
+        <v>23</v>
+      </c>
+      <c r="S47" t="n">
+        <v>1.8334</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -25458,6 +26916,18 @@
       <c r="O48" t="n">
         <v>0</v>
       </c>
+      <c r="P48" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.0426</v>
+      </c>
+      <c r="R48" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="S48" t="n">
+        <v>1.857</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -25505,6 +26975,18 @@
       <c r="O49" t="n">
         <v>0</v>
       </c>
+      <c r="P49" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.0164</v>
+      </c>
+      <c r="R49" t="n">
+        <v>24</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.8455</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -25552,6 +27034,18 @@
       <c r="O50" t="n">
         <v>0</v>
       </c>
+      <c r="P50" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>1.9906</v>
+      </c>
+      <c r="R50" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="S50" t="n">
+        <v>1.8286</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -25599,6 +27093,18 @@
       <c r="O51" t="n">
         <v>0</v>
       </c>
+      <c r="P51" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>1.9822</v>
+      </c>
+      <c r="R51" t="n">
+        <v>25</v>
+      </c>
+      <c r="S51" t="n">
+        <v>1.8244</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -25646,6 +27152,18 @@
       <c r="O52" t="n">
         <v>0</v>
       </c>
+      <c r="P52" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>1.9423</v>
+      </c>
+      <c r="R52" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1.8117</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -25693,6 +27211,18 @@
       <c r="O53" t="n">
         <v>0</v>
       </c>
+      <c r="P53" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>1.9356</v>
+      </c>
+      <c r="R53" t="n">
+        <v>26</v>
+      </c>
+      <c r="S53" t="n">
+        <v>1.7918</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -25740,6 +27270,18 @@
       <c r="O54" t="n">
         <v>0</v>
       </c>
+      <c r="P54" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>1.9071</v>
+      </c>
+      <c r="R54" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="S54" t="n">
+        <v>1.7651</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -25787,6 +27329,18 @@
       <c r="O55" t="n">
         <v>0</v>
       </c>
+      <c r="P55" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>1.9798</v>
+      </c>
+      <c r="R55" t="n">
+        <v>27</v>
+      </c>
+      <c r="S55" t="n">
+        <v>1.7993</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -25834,6 +27388,18 @@
       <c r="O56" t="n">
         <v>0</v>
       </c>
+      <c r="P56" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>2.0438</v>
+      </c>
+      <c r="R56" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="S56" t="n">
+        <v>1.8373</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -25881,6 +27447,18 @@
       <c r="O57" t="n">
         <v>0</v>
       </c>
+      <c r="P57" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>2.052</v>
+      </c>
+      <c r="R57" t="n">
+        <v>28</v>
+      </c>
+      <c r="S57" t="n">
+        <v>1.8228</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -25928,6 +27506,18 @@
       <c r="O58" t="n">
         <v>0</v>
       </c>
+      <c r="P58" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>2.0002</v>
+      </c>
+      <c r="R58" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="S58" t="n">
+        <v>1.8322</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -25975,6 +27565,18 @@
       <c r="O59" t="n">
         <v>0</v>
       </c>
+      <c r="P59" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1.9915</v>
+      </c>
+      <c r="R59" t="n">
+        <v>29</v>
+      </c>
+      <c r="S59" t="n">
+        <v>1.8125</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -26022,6 +27624,18 @@
       <c r="O60" t="n">
         <v>0</v>
       </c>
+      <c r="P60" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>1.9348</v>
+      </c>
+      <c r="R60" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="S60" t="n">
+        <v>1.8126</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -26069,6 +27683,18 @@
       <c r="O61" t="n">
         <v>0</v>
       </c>
+      <c r="P61" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>2.0975</v>
+      </c>
+      <c r="R61" t="n">
+        <v>30</v>
+      </c>
+      <c r="S61" t="n">
+        <v>1.8336</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -26116,6 +27742,18 @@
       <c r="O62" t="n">
         <v>0</v>
       </c>
+      <c r="P62" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>3.9331</v>
+      </c>
+      <c r="R62" t="n">
+        <v>30.52</v>
+      </c>
+      <c r="S62" t="n">
+        <v>2.7276</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -26163,6 +27801,18 @@
       <c r="O63" t="n">
         <v>0</v>
       </c>
+      <c r="P63" t="n">
+        <v>31</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>4.2052</v>
+      </c>
+      <c r="R63" t="n">
+        <v>31.02</v>
+      </c>
+      <c r="S63" t="n">
+        <v>3.0275</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -26210,6 +27860,18 @@
       <c r="O64" t="n">
         <v>0</v>
       </c>
+      <c r="P64" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>4.1181</v>
+      </c>
+      <c r="R64" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="S64" t="n">
+        <v>3.0034</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -26257,6 +27919,18 @@
       <c r="O65" t="n">
         <v>0</v>
       </c>
+      <c r="P65" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>4.0365</v>
+      </c>
+      <c r="R65" t="n">
+        <v>32.02</v>
+      </c>
+      <c r="S65" t="n">
+        <v>3.0173</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -26304,6 +27978,18 @@
       <c r="O66" t="n">
         <v>0</v>
       </c>
+      <c r="P66" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>3.9786</v>
+      </c>
+      <c r="R66" t="n">
+        <v>32.52</v>
+      </c>
+      <c r="S66" t="n">
+        <v>3.0106</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -26351,6 +28037,18 @@
       <c r="O67" t="n">
         <v>0</v>
       </c>
+      <c r="P67" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>3.9204</v>
+      </c>
+      <c r="R67" t="n">
+        <v>33.02</v>
+      </c>
+      <c r="S67" t="n">
+        <v>2.987</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -26398,6 +28096,18 @@
       <c r="O68" t="n">
         <v>0</v>
       </c>
+      <c r="P68" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="R68" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="S68" t="n">
+        <v>2.9736</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -26445,6 +28155,18 @@
       <c r="O69" t="n">
         <v>0</v>
       </c>
+      <c r="P69" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>3.8439</v>
+      </c>
+      <c r="R69" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="S69" t="n">
+        <v>2.9626</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -26492,6 +28214,18 @@
       <c r="O70" t="n">
         <v>0</v>
       </c>
+      <c r="P70" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>3.8084</v>
+      </c>
+      <c r="R70" t="n">
+        <v>34.52</v>
+      </c>
+      <c r="S70" t="n">
+        <v>2.9477</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -26539,6 +28273,18 @@
       <c r="O71" t="n">
         <v>0</v>
       </c>
+      <c r="P71" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>3.7804</v>
+      </c>
+      <c r="R71" t="n">
+        <v>35.02</v>
+      </c>
+      <c r="S71" t="n">
+        <v>2.9339</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -26586,6 +28332,18 @@
       <c r="O72" t="n">
         <v>0</v>
       </c>
+      <c r="P72" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>3.7484</v>
+      </c>
+      <c r="R72" t="n">
+        <v>35.52</v>
+      </c>
+      <c r="S72" t="n">
+        <v>2.9199</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -26633,6 +28391,18 @@
       <c r="O73" t="n">
         <v>0</v>
       </c>
+      <c r="P73" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>3.7064</v>
+      </c>
+      <c r="R73" t="n">
+        <v>36.02</v>
+      </c>
+      <c r="S73" t="n">
+        <v>2.9061</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -26680,6 +28450,18 @@
       <c r="O74" t="n">
         <v>0</v>
       </c>
+      <c r="P74" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>3.6717</v>
+      </c>
+      <c r="R74" t="n">
+        <v>36.52</v>
+      </c>
+      <c r="S74" t="n">
+        <v>2.8722</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -26727,6 +28509,18 @@
       <c r="O75" t="n">
         <v>0</v>
       </c>
+      <c r="P75" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>3.6484</v>
+      </c>
+      <c r="R75" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="S75" t="n">
+        <v>2.8736</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -26774,6 +28568,18 @@
       <c r="O76" t="n">
         <v>0</v>
       </c>
+      <c r="P76" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>3.6148</v>
+      </c>
+      <c r="R76" t="n">
+        <v>37.52</v>
+      </c>
+      <c r="S76" t="n">
+        <v>2.8601</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -26821,6 +28627,18 @@
       <c r="O77" t="n">
         <v>0</v>
       </c>
+      <c r="P77" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>3.5859</v>
+      </c>
+      <c r="R77" t="n">
+        <v>38.02</v>
+      </c>
+      <c r="S77" t="n">
+        <v>2.8423</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -26868,6 +28686,18 @@
       <c r="O78" t="n">
         <v>0</v>
       </c>
+      <c r="P78" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>3.5456</v>
+      </c>
+      <c r="R78" t="n">
+        <v>38.52</v>
+      </c>
+      <c r="S78" t="n">
+        <v>2.8367</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -26915,6 +28745,18 @@
       <c r="O79" t="n">
         <v>0</v>
       </c>
+      <c r="P79" t="n">
+        <v>39</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>3.5065</v>
+      </c>
+      <c r="R79" t="n">
+        <v>39.02</v>
+      </c>
+      <c r="S79" t="n">
+        <v>2.8382</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -26962,6 +28804,18 @@
       <c r="O80" t="n">
         <v>0</v>
       </c>
+      <c r="P80" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>3.4809</v>
+      </c>
+      <c r="R80" t="n">
+        <v>39.52</v>
+      </c>
+      <c r="S80" t="n">
+        <v>2.8279</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -27009,6 +28863,18 @@
       <c r="O81" t="n">
         <v>0</v>
       </c>
+      <c r="P81" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>3.4522</v>
+      </c>
+      <c r="R81" t="n">
+        <v>40.02</v>
+      </c>
+      <c r="S81" t="n">
+        <v>2.8273</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -27056,6 +28922,18 @@
       <c r="O82" t="n">
         <v>0</v>
       </c>
+      <c r="P82" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>3.4358</v>
+      </c>
+      <c r="R82" t="n">
+        <v>40.52</v>
+      </c>
+      <c r="S82" t="n">
+        <v>2.8211</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -27103,6 +28981,18 @@
       <c r="O83" t="n">
         <v>0</v>
       </c>
+      <c r="P83" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>3.419</v>
+      </c>
+      <c r="R83" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="S83" t="n">
+        <v>2.8089</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -27150,6 +29040,18 @@
       <c r="O84" t="n">
         <v>0</v>
       </c>
+      <c r="P84" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>3.4024</v>
+      </c>
+      <c r="R84" t="n">
+        <v>41.52</v>
+      </c>
+      <c r="S84" t="n">
+        <v>2.7976</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -27197,6 +29099,18 @@
       <c r="O85" t="n">
         <v>0</v>
       </c>
+      <c r="P85" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>3.3844</v>
+      </c>
+      <c r="R85" t="n">
+        <v>42.02</v>
+      </c>
+      <c r="S85" t="n">
+        <v>2.7931</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -27244,6 +29158,18 @@
       <c r="O86" t="n">
         <v>0</v>
       </c>
+      <c r="P86" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>3.3664</v>
+      </c>
+      <c r="R86" t="n">
+        <v>42.52</v>
+      </c>
+      <c r="S86" t="n">
+        <v>2.7843</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -27291,6 +29217,18 @@
       <c r="O87" t="n">
         <v>0</v>
       </c>
+      <c r="P87" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>3.3447</v>
+      </c>
+      <c r="R87" t="n">
+        <v>43.02</v>
+      </c>
+      <c r="S87" t="n">
+        <v>2.783</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -27338,6 +29276,18 @@
       <c r="O88" t="n">
         <v>0</v>
       </c>
+      <c r="P88" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>3.3243</v>
+      </c>
+      <c r="R88" t="n">
+        <v>43.52</v>
+      </c>
+      <c r="S88" t="n">
+        <v>2.7763</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -27385,6 +29335,18 @@
       <c r="O89" t="n">
         <v>0</v>
       </c>
+      <c r="P89" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>3.3053</v>
+      </c>
+      <c r="R89" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="S89" t="n">
+        <v>2.7702</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -27431,6 +29393,18 @@
       </c>
       <c r="O90" t="n">
         <v>1</v>
+      </c>
+      <c r="P90" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>3.2804</v>
+      </c>
+      <c r="R90" t="n">
+        <v>44.52</v>
+      </c>
+      <c r="S90" t="n">
+        <v>2.7605</v>
       </c>
     </row>
     <row r="91">

</xml_diff>

<commit_message>
Fig.7: CAT-47 line removed (process figure compares with default/robust; CAT-47 stays in result tables and sheet columns C-D)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7.xlsx
+++ b/figs/data/fig7.xlsx
@@ -234,42 +234,6 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'OLTP→Varmail'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
-              <a:solidFill>
-                <a:srgbClr val="1D1D1F"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'OLTP→Varmail'!$C$2:$C$60</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'OLTP→Varmail'!$D$2:$D$60</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
               <f>'OLTP→Varmail'!B1</f>
             </strRef>
           </tx>
@@ -302,8 +266,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="4"/>
-          <order val="4"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'OLTP→Varmail'!X1</f>
@@ -840,42 +804,6 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'FIO-Fast→Varmail'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
-              <a:solidFill>
-                <a:srgbClr val="1D1D1F"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'FIO-Fast→Varmail'!$C$2:$C$90</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'FIO-Fast→Varmail'!$D$2:$D$90</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
               <f>'FIO-Fast→Varmail'!B1</f>
             </strRef>
           </tx>
@@ -908,8 +836,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="4"/>
-          <order val="4"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'FIO-Fast→Varmail'!X1</f>

</xml_diff>